<commit_message>
feat(F-NAR-019): polish TREE-DIF-008 xlsx
Alignement xlsx sur merged vocal après re-apply.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-008.xlsx
+++ b/stories/arbres/TREE-DIF-008.xlsx
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La goutte grossit au bord de la toile. Elle tremble, puis choisit le bois de l'étal. Un grain de cannelle s'y colle, brun et minuscule. Le marché assemble ses caisses, sans crier. Ça sent l'écorce mouillée, et le fruit coupé. Tu as vu ce grain, Raphaël ? Il est coincé dans l'eau. La toile va goutter longtemps. Une caisse glisse sur le bois mouillé. Raphaël la rattrape des deux mains. Merci, tu as tenu la caisse. Je tiens le stand, moi. Un fruit, pour Mila, tout de suite. En ce moment, Raphaël avance le bras vers elle. Mila arrive, les mains au fond des poches. Viens, c'est pour toi ! Mila ne dit rien. Ses doigts restent cachés. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Papa s'accroupit, à la hauteur des deux. Tu l'as vue, ses poches ? Elle n'a rien dit. Ses mains sont restées dedans.</t>
+          <t>La goutte grossit au bord de la toile. Elle tremble, puis choisit le bois de l'étal. Un grain de cannelle s'y colle, brun et minuscule. Il pique un peu, collé au bois mouillé. Le marché assemble ses caisses, sans crier. Des voix s'installent, plus loin, pas ici. Ça sent l'écorce mouillée, et le fruit coupé. Tu as vu ce grain, Raphaël ? Il est coincé dans l'eau. La toile va goutter longtemps. Une caisse glisse sur le bois mouillé. Raphaël la rattrape des deux mains. Merci, tu as tenu la caisse. Je tiens le stand, moi. Un fruit, pour Mila, tout de suite. En ce moment, Raphaël avance le bras vers elle. Mila arrive, les mains au fond des poches. Viens, c'est pour toi ! Mila ne dit rien. Ses doigts restent cachés. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Papa s'accroupit, à la hauteur des deux. Tu l'as vue, ses poches ? Elle n'a rien dit. Ses mains sont restées dedans.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La goutte grossit au bord de la toile. Elle tremble, puis choisit le bois de l'étal. Un &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; s'y colle, brun et minuscule. Le marché assemble ses caisses, sans crier. Ça sent l'écorce mouillée, et le fruit coupé. Tu as vu ce grain, Raphaël ? Il est coincé dans l'eau. La toile va goutter longtemps. Une caisse glisse sur le bois mouillé. Raphaël la rattrape des deux mains. Merci, tu as tenu la caisse. Je tiens le stand, moi. Un fruit, pour Mila, tout de suite. En ce moment, Raphaël avance le bras vers elle. Mila arrive, les mains au fond des poches. Viens, c'est pour toi ! Mila ne dit rien. Ses doigts restent cachés. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Papa s'accroupit, à la hauteur des deux. Tu l'as vue, ses poches ? Elle n'a rien dit. Ses mains sont restées dedans.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La goutte grossit au bord de la toile. Elle tremble, puis choisit le bois de l'étal. Un &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; s'y colle, brun et minuscule. Il pique un peu, collé au bois mouillé. Le marché assemble ses caisses, sans crier. Des voix s'installent, plus loin, pas ici. Ça sent l'écorce mouillée, et le fruit coupé. Tu as vu ce grain, Raphaël ? Il est coincé dans l'eau. La toile va goutter longtemps. Une caisse glisse sur le bois mouillé. Raphaël la rattrape des deux mains. Merci, tu as tenu la caisse. Je tiens le stand, moi. Un fruit, pour Mila, tout de suite. En ce moment, Raphaël avance le bras vers elle. Mila arrive, les mains au fond des poches. Viens, c'est pour toi ! Mila ne dit rien. Ses doigts restent cachés. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Papa s'accroupit, à la hauteur des deux. Tu l'as vue, ses poches ? Elle n'a rien dit. Ses mains sont restées dedans.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>La goutte grossit au bord de la toile. Elle tremble, puis choisit le bois de l'étal. Un &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; s'y colle, brun et minuscule. Le marché assemble ses caisses, sans crier. Ça sent l'écorce mouillée, et le fruit coupé. Tu as vu ce grain, Raphaël ? Il est coincé dans l'eau. La toile va goutter longtemps. Une caisse glisse sur le bois mouillé. Raphaël la rattrape des deux mains. Merci, tu as tenu la caisse. Je tiens le stand, moi. Un fruit, pour Mila, tout de suite. En ce moment, Raphaël avance le bras vers elle. Mila arrive, les mains au fond des poches. Viens, c'est pour toi ! Mila ne dit rien. Ses doigts restent cachés. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Papa s'accroupit, à la hauteur des deux. Tu l'as vue, ses poches ? Elle n'a rien dit. Ses mains sont restées dedans. [pause]</t>
+          <t>La goutte grossit au bord de la toile. Elle tremble, puis choisit le bois de l'étal. Un &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; s'y colle, brun et minuscule. Il pique un peu, collé au bois mouillé. Le marché assemble ses caisses, sans crier. Des voix s'installent, plus loin, pas ici. Ça sent l'écorce mouillée, et le fruit coupé. Tu as vu ce grain, Raphaël ? Il est coincé dans l'eau. La toile va goutter longtemps. Une caisse glisse sur le bois mouillé. Raphaël la rattrape des deux mains. Merci, tu as tenu la caisse. Je tiens le stand, moi. Un fruit, pour Mila, tout de suite. En ce moment, Raphaël avance le bras vers elle. Mila arrive, les mains au fond des poches. Viens, c'est pour toi ! Mila ne dit rien. Ses doigts restent cachés. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Papa s'accroupit, à la hauteur des deux. Tu l'as vue, ses poches ? Elle n'a rien dit. Ses mains sont restées dedans. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1344,7 +1344,9 @@
           <t>narrateur|La goutte grossit au bord de la toile.
 narrateur|Elle tremble, puis choisit le bois de l'étal.
 narrateur|Un grain de cannelle s'y colle, brun et minuscule.
+narrateur|Il pique un peu, collé au bois mouillé.
 narrateur|Le marché assemble ses caisses, sans crier.
+narrateur|Des voix s'installent, plus loin, pas ici.
 narrateur|Ça sent l'écorce mouillée, et le fruit coupé.
 papa|Tu as vu ce grain, Raphaël ?
 enfant-m|Il est coincé dans l'eau.
@@ -1598,17 +1600,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël glisse sous le store jaune. La toile jette des ronds d'or sur les citrons. Ils sentent le zeste, fort. La balance, le sac et la caisse restent là. Il cueille un citron, trop vite. Prends, Mila ! Mila recule d'un pas. Le citron reste seul, dans sa paume. Le sourire de Raphaël se plie. Elle n'a pas tendu les doigts. Maman s'accroupit, près des caisses jaunes. Une goutte dorée tremble au bord de la toile. Elle tombe près du grain de cannelle. Le grain est mouillé. Tu le vois, sur le bois ?</t>
+          <t>Raphaël glisse sous le store jaune. La toile jette des ronds d'or sur les citrons. Ils sentent le zeste, fort. La balance, le sac et la caisse restent là. Il cueille un citron, trop vite. Prends, Mila ! Mila recule d'un pas. Le citron reste seul, dans sa paume. Le sourire de Raphaël se plie. Elle n'a pas tendu les doigts. Maman s'accroupit, près des caisses jaunes. Une goutte dorée tremble au bord de la toile. Elle tombe près du grain de cannelle. Le grain est mouillé. Tu le vois, sur le bois ? Un client passe, sans s'arrêter.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël glisse sous le &lt;emphasis level="moderate"&gt;store jaune&lt;/emphasis&gt;. La toile jette des ronds d'or sur les citrons. Ils sentent le zeste, fort. La balance, le sac et la caisse restent là. Il cueille un citron, trop vite. Prends, Mila ! Mila recule d'un pas. Le citron reste seul, dans sa paume. Le sourire de Raphaël se plie. Elle n'a pas tendu les doigts. Maman s'accroupit, près des caisses jaunes. Une goutte dorée tremble au bord de la toile. Elle tombe près du grain de cannelle. Le grain est mouillé. Tu le vois, sur le bois ?&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël glisse sous le &lt;emphasis level="moderate"&gt;store jaune&lt;/emphasis&gt;. La toile jette des ronds d'or sur les citrons. Ils sentent le zeste, fort. La balance, le sac et la caisse restent là. Il cueille un citron, trop vite. Prends, Mila ! Mila recule d'un pas. Le citron reste seul, dans sa paume. Le sourire de Raphaël se plie. Elle n'a pas tendu les doigts. Maman s'accroupit, près des caisses jaunes. Une goutte dorée tremble au bord de la toile. Elle tombe près du grain de cannelle. Le grain est mouillé. Tu le vois, sur le bois ? Un client passe, sans s'arrêter.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël glisse sous le &lt;emphasis&gt;store jaune&lt;/emphasis&gt;. La toile jette des ronds d'or sur les citrons. Ils sentent le zeste, fort. La balance, le sac et la caisse restent là. Il cueille un citron, trop vite. Prends, Mila ! Mila recule d'un pas. Le citron reste seul, dans sa paume. Le sourire de Raphaël se plie. Elle n'a pas tendu les doigts. Maman s'accroupit, près des caisses jaunes. Une goutte dorée tremble au bord de la toile. Elle tombe près du grain de cannelle. Le grain est mouillé. Tu le vois, sur le bois ? [pause]</t>
+          <t>Raphaël glisse sous le &lt;emphasis&gt;store jaune&lt;/emphasis&gt;. La toile jette des ronds d'or sur les citrons. Ils sentent le zeste, fort. La balance, le sac et la caisse restent là. Il cueille un citron, trop vite. Prends, Mila ! Mila recule d'un pas. Le citron reste seul, dans sa paume. Le sourire de Raphaël se plie. Elle n'a pas tendu les doigts. Maman s'accroupit, près des caisses jaunes. Une goutte dorée tremble au bord de la toile. Elle tombe près du grain de cannelle. Le grain est mouillé. Tu le vois, sur le bois ? Un client passe, sans s'arrêter. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1756,7 +1758,8 @@
 narrateur|Une goutte dorée tremble au bord de la toile.
 narrateur|Elle tombe près du grain de cannelle.
 enfant-m|Le grain est mouillé.
-papa|Tu le vois, sur le bois ?</t>
+papa|Tu le vois, sur le bois ?
+narrateur|Un client passe, sans s'arrêter.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -2928,17 +2931,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Le stand a failli rester sans regard. Mila est restée au bord, les yeux ouverts. Tu as regardé le chiffre. Oui. L'aiguille ne danse plus. Le citron a gardé sa place. La goutte jaune a séché en croissant mince. Le grain de cannelle tient sur le plateau froid.</t>
+          <t>Le stand a failli rester sans regard. Mila est restée au bord, les yeux ouverts. Tu as regardé le chiffre. Oui. L'aiguille ne danse plus. Le citron a gardé sa place. La goutte jaune a séché en trait d'or. Le grain de cannelle tient sur le plateau froid.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le stand a failli rester sans regard. Mila est restée au bord, les yeux ouverts. Tu as regardé le chiffre. Oui. L'aiguille ne danse plus. Le citron a gardé sa place. La goutte jaune a séché en croissant mince. Le &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; tient sur le plateau froid.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le stand a failli rester sans regard. Mila est restée au bord, les yeux ouverts. Tu as regardé le chiffre. Oui. L'aiguille ne danse plus. Le citron a gardé sa place. La goutte jaune a séché en trait d'or. Le &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; tient sur le plateau froid.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le stand a failli rester sans regard. Mila est restée au bord, les yeux ouverts. Tu as regardé le chiffre. Oui. L'aiguille ne danse plus. Le citron a gardé sa place. La goutte jaune a séché en croissant mince. Le &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; tient sur le plateau froid.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le stand a failli rester sans regard. Mila est restée au bord, les yeux ouverts. Tu as regardé le chiffre. Oui. L'aiguille ne danse plus. Le citron a gardé sa place. La goutte jaune a séché en trait d'or. Le &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; tient sur le plateau froid.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -3082,7 +3085,7 @@
 enfant-f|Oui.
 papa|L'aiguille ne danse plus.
 maman|Le citron a gardé sa place.
-narrateur|La goutte jaune a séché en croissant mince.
+narrateur|La goutte jaune a séché en trait d'or.
 narrateur|Le grain de cannelle tient sur le plateau froid.</t>
         </is>
       </c>
@@ -3298,17 +3301,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Mila revient, les joues un peu chaudes. Maintenant ? Oui. C'est pour toi. Elle s'approche de la balance. Vous avez pris le temps. La goutte jaune n'est plus qu'un trait. Le citron attend, et le grain brille à côté.</t>
+          <t>Mila revient, les joues un peu chaudes. Maintenant ? Oui. C'est pour toi. Elle s'approche de la balance. Vous avez pris le temps. La goutte jaune n'est plus qu'un trait. Le citron attend, et le grain de cannelle brille à côté.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, les joues un peu chaudes. Maintenant ? Oui. C'est pour toi. Elle s'approche de la balance. Vous avez pris le temps. La goutte jaune n'est plus qu'un trait. Le citron attend, et le grain brille à côté.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, les joues un peu chaudes. Maintenant ? Oui. C'est pour toi. Elle s'approche de la balance. Vous avez pris le temps. La goutte jaune n'est plus qu'un trait. Le citron attend, et le &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; brille à côté.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, les joues un peu chaudes. Maintenant ? Oui. C'est pour toi. Elle s'approche de la balance. Vous avez pris le temps. La goutte jaune n'est plus qu'un trait. Le citron attend, et le grain brille à côté.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, les joues un peu chaudes. Maintenant ? Oui. C'est pour toi. Elle s'approche de la balance. Vous avez pris le temps. La goutte jaune n'est plus qu'un trait. Le citron attend, et le &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; brille à côté.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3453,7 +3456,7 @@
 narrateur|Elle s'approche de la balance.
 papa|Vous avez pris le temps.
 narrateur|La goutte jaune n'est plus qu'un trait.
-narrateur|Le citron attend, et le grain brille à côté.</t>
+narrateur|Le citron attend, et le grain de cannelle brille à côté.</t>
         </is>
       </c>
       <c r="AX13" t="inlineStr">
@@ -3668,17 +3671,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Le citron a failli rouler, tout à l'heure. On l'a pesé. Le stand est à nous. Vous avez offert le fruit. Le métal a deux traces de doigts. La goutte jaune a quitté le zeste. Le bois de l'étal redevient sec. Deux doigts ont coincé le grain entre le métal et le zeste.</t>
+          <t>Le citron a failli rouler, tout à l'heure. On l'a pesé. Le stand est à nous. Vous avez offert le fruit. Le métal a deux traces de doigts. La goutte jaune a quitté le zeste. Le bois de l'étal redevient sec. Deux doigts ont coincé le grain de cannelle entre métal et zeste.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le citron a failli rouler, tout à l'heure. On l'a pesé. Le stand est à nous. Vous avez offert le fruit. Le métal a deux traces de doigts. La goutte jaune a quitté le zeste. Le bois de l'étal redevient sec. Deux doigts ont coincé le grain entre le métal et le zeste.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le citron a failli rouler, tout à l'heure. On l'a pesé. Le stand est à nous. Vous avez offert le fruit. Le métal a deux traces de doigts. La goutte jaune a quitté le zeste. Le bois de l'étal redevient sec. Deux doigts ont coincé le &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; entre métal et zeste.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le citron a failli rouler, tout à l'heure. On l'a pesé. Le stand est à nous. Vous avez offert le fruit. Le métal a deux traces de doigts. La goutte jaune a quitté le zeste. Le bois de l'étal redevient sec. Deux doigts ont coincé le grain entre le métal et le zeste.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le citron a failli rouler, tout à l'heure. On l'a pesé. Le stand est à nous. Vous avez offert le fruit. Le métal a deux traces de doigts. La goutte jaune a quitté le zeste. Le bois de l'étal redevient sec. Deux doigts ont coincé le &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; entre métal et zeste.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -3823,7 +3826,7 @@
 maman|Le métal a deux traces de doigts.
 narrateur|La goutte jaune a quitté le zeste.
 narrateur|Le bois de l'étal redevient sec.
-narrateur|Deux doigts ont coincé le grain entre le métal et le zeste.</t>
+narrateur|Deux doigts ont coincé le grain de cannelle entre métal et zeste.</t>
         </is>
       </c>
       <c r="AX15" t="inlineStr">
@@ -4428,17 +4431,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Le sac a failli se fermer trop tôt. Mila reste au bord, le nez sur le papier. Tu as regardé le fond. Oui. Le papier est resté ouvert. Le zeste habite le brun. La goutte jaune a séché sur le pli. Le sac brun garde une ombre de citron, et le grain.</t>
+          <t>Le sac a failli se fermer trop tôt. Mila reste au bord, le nez sur le papier. Tu as regardé le fond. Oui. Le papier est resté ouvert. Le zeste habite le brun. La goutte jaune a séché sur le pli. Le sac brun garde une ombre de citron, et le grain de cannelle.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le sac a failli se fermer trop tôt. Mila reste au bord, le nez sur le papier. Tu as regardé le fond. Oui. Le papier est resté ouvert. Le zeste habite le brun. La goutte jaune a séché sur le pli. Le sac brun garde une ombre de citron, et le grain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le sac a failli se fermer trop tôt. Mila reste au bord, le nez sur le papier. Tu as regardé le fond. Oui. Le papier est resté ouvert. Le zeste habite le brun. La goutte jaune a séché sur le pli. Le sac brun garde une ombre de citron, et le &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le sac a failli se fermer trop tôt. Mila reste au bord, le nez sur le papier. Tu as regardé le fond. Oui. Le papier est resté ouvert. Le zeste habite le brun. La goutte jaune a séché sur le pli. Le sac brun garde une ombre de citron, et le grain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le sac a failli se fermer trop tôt. Mila reste au bord, le nez sur le papier. Tu as regardé le fond. Oui. Le papier est resté ouvert. Le zeste habite le brun. La goutte jaune a séché sur le pli. Le sac brun garde une ombre de citron, et le &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt;.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4583,7 +4586,7 @@
 papa|Le papier est resté ouvert.
 maman|Le zeste habite le brun.
 narrateur|La goutte jaune a séché sur le pli.
-narrateur|Le sac brun garde une ombre de citron, et le grain.</t>
+narrateur|Le sac brun garde une ombre de citron, et le grain de cannelle.</t>
         </is>
       </c>
       <c r="AX19" t="inlineStr">
@@ -4798,17 +4801,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Mila revient, un sac d'un autre étal à la main. Maintenant ? Oui, le tien est là. Elle s'approche du papier. Vous avez pris le temps. Le sac l'attendait. La goutte jaune a quitté le col. Le papier reste ouvert, le grain au bord.</t>
+          <t>Mila revient, un sac d'un autre étal à la main. Maintenant ? Oui, le tien est là. Elle s'approche du papier. Vous avez pris le temps. Le sac l'attendait. La goutte jaune a quitté le col. Le papier reste ouvert, le grain de cannelle au bord.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, un sac d'un autre étal à la main. Maintenant ? Oui, le tien est là. Elle s'approche du papier. Vous avez pris le temps. Le sac l'attendait. La goutte jaune a quitté le col. Le papier reste ouvert, le grain au bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, un sac d'un autre étal à la main. Maintenant ? Oui, le tien est là. Elle s'approche du papier. Vous avez pris le temps. Le sac l'attendait. La goutte jaune a quitté le col. Le papier reste ouvert, le &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; au bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, un sac d'un autre étal à la main. Maintenant ? Oui, le tien est là. Elle s'approche du papier. Vous avez pris le temps. Le sac l'attendait. La goutte jaune a quitté le col. Le papier reste ouvert, le grain au bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, un sac d'un autre étal à la main. Maintenant ? Oui, le tien est là. Elle s'approche du papier. Vous avez pris le temps. Le sac l'attendait. La goutte jaune a quitté le col. Le papier reste ouvert, le &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; au bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -4953,7 +4956,7 @@
 papa|Vous avez pris le temps.
 maman|Le sac l'attendait.
 narrateur|La goutte jaune a quitté le col.
-narrateur|Le papier reste ouvert, le grain au bord.</t>
+narrateur|Le papier reste ouvert, le grain de cannelle au bord.</t>
         </is>
       </c>
       <c r="AX21" t="inlineStr">
@@ -5168,17 +5171,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Le papier a failli se fendre jusqu'au bout. On l'a porté. Le stand est à nous. Vous avez offert le fruit. Le sac penche entre deux petites mains. La goutte jaune a séché dans le fond. Le bois de l'étal redevient sec. Le sac penche entre deux petites mains, grain au fond.</t>
+          <t>Le papier a failli se fendre jusqu'au bout. On l'a porté. Le stand est à nous. Vous avez offert le fruit. Le sac penche entre deux petites mains. La goutte jaune a séché dans le fond. Le bois de l'étal redevient sec. Le sac penche entre deux petites mains, grain de cannelle au fond.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le papier a failli se fendre jusqu'au bout. On l'a porté. Le stand est à nous. Vous avez offert le fruit. Le sac penche entre deux petites mains. La goutte jaune a séché dans le fond. Le bois de l'étal redevient sec. Le sac penche entre deux petites mains, grain au fond.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le papier a failli se fendre jusqu'au bout. On l'a porté. Le stand est à nous. Vous avez offert le fruit. Le sac penche entre deux petites mains. La goutte jaune a séché dans le fond. Le bois de l'étal redevient sec. Le sac penche entre deux petites mains, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; au fond.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le papier a failli se fendre jusqu'au bout. On l'a porté. Le stand est à nous. Vous avez offert le fruit. Le sac penche entre deux petites mains. La goutte jaune a séché dans le fond. Le bois de l'étal redevient sec. Le sac penche entre deux petites mains, grain au fond.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le papier a failli se fendre jusqu'au bout. On l'a porté. Le stand est à nous. Vous avez offert le fruit. Le sac penche entre deux petites mains. La goutte jaune a séché dans le fond. Le bois de l'étal redevient sec. Le sac penche entre deux petites mains, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; au fond.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -5323,7 +5326,7 @@
 maman|Le sac penche entre deux petites mains.
 narrateur|La goutte jaune a séché dans le fond.
 narrateur|Le bois de l'étal redevient sec.
-narrateur|Le sac penche entre deux petites mains, grain au fond.</t>
+narrateur|Le sac penche entre deux petites mains, grain de cannelle au fond.</t>
         </is>
       </c>
       <c r="AX23" t="inlineStr">
@@ -5928,17 +5931,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>La tour a failli tout emporter. Mila reste au bord, les yeux sur le bas. Tu as regardé en bas. Oui. Les citrons du haut brillent, trop loin. Le bois d'en bas est à sa hauteur. La goutte jaune a séché sur la planche. Les citrons du haut brillent, grain sur le bord.</t>
+          <t>La tour a failli tout emporter. Mila reste au bord, les yeux sur le bas. Tu as regardé en bas. Oui. Les citrons du haut brillent, trop loin. Le bois d'en bas est à sa hauteur. La goutte jaune a séché sur la planche. Les citrons du haut brillent, grain de cannelle sur le bord.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La tour a failli tout emporter. Mila reste au bord, les yeux sur le bas. Tu as regardé en bas. Oui. Les citrons du haut brillent, trop loin. Le bois d'en bas est à sa hauteur. La goutte jaune a séché sur la planche. Les citrons du haut brillent, grain sur le bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La tour a failli tout emporter. Mila reste au bord, les yeux sur le bas. Tu as regardé en bas. Oui. Les citrons du haut brillent, trop loin. Le bois d'en bas est à sa hauteur. La goutte jaune a séché sur la planche. Les citrons du haut brillent, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; sur le bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La tour a failli tout emporter. Mila reste au bord, les yeux sur le bas. Tu as regardé en bas. Oui. Les citrons du haut brillent, trop loin. Le bois d'en bas est à sa hauteur. La goutte jaune a séché sur la planche. Les citrons du haut brillent, grain sur le bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La tour a failli tout emporter. Mila reste au bord, les yeux sur le bas. Tu as regardé en bas. Oui. Les citrons du haut brillent, trop loin. Le bois d'en bas est à sa hauteur. La goutte jaune a séché sur la planche. Les citrons du haut brillent, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; sur le bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -6083,7 +6086,7 @@
 papa|Les citrons du haut brillent, trop loin.
 maman|Le bois d'en bas est à sa hauteur.
 narrateur|La goutte jaune a séché sur la planche.
-narrateur|Les citrons du haut brillent, grain sur le bord.</t>
+narrateur|Les citrons du haut brillent, grain de cannelle sur le bord.</t>
         </is>
       </c>
       <c r="AX27" t="inlineStr">
@@ -6298,17 +6301,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Mila revient, les poches un peu moins profondes. Maintenant ? Oui, ta place est là. Elle s'approche de la caisse. Vous avez pris le temps. La place vide l'attendait. La goutte jaune a quitté le bord. Une place vide reste, le grain posé dessus.</t>
+          <t>Mila revient, les poches un peu moins profondes. Maintenant ? Oui, ta place est là. Elle s'approche de la caisse. Vous avez pris le temps. La place vide l'attendait. La goutte jaune a quitté le bord. Une place vide reste, le grain de cannelle posé dessus.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, les poches un peu moins profondes. Maintenant ? Oui, ta place est là. Elle s'approche de la caisse. Vous avez pris le temps. La place vide l'attendait. La goutte jaune a quitté le bord. Une place vide reste, le grain posé dessus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, les poches un peu moins profondes. Maintenant ? Oui, ta place est là. Elle s'approche de la caisse. Vous avez pris le temps. La place vide l'attendait. La goutte jaune a quitté le bord. Une place vide reste, le &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; posé dessus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, les poches un peu moins profondes. Maintenant ? Oui, ta place est là. Elle s'approche de la caisse. Vous avez pris le temps. La place vide l'attendait. La goutte jaune a quitté le bord. Une place vide reste, le grain posé dessus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, les poches un peu moins profondes. Maintenant ? Oui, ta place est là. Elle s'approche de la caisse. Vous avez pris le temps. La place vide l'attendait. La goutte jaune a quitté le bord. Une place vide reste, le &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; posé dessus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -6453,7 +6456,7 @@
 papa|Vous avez pris le temps.
 maman|La place vide l'attendait.
 narrateur|La goutte jaune a quitté le bord.
-narrateur|Une place vide reste, le grain posé dessus.</t>
+narrateur|Une place vide reste, le grain de cannelle posé dessus.</t>
         </is>
       </c>
       <c r="AX29" t="inlineStr">
@@ -6668,17 +6671,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Le citron a failli tomber de la tour. On l'a rangé. Le stand est à nous. Vous avez offert le fruit. La tour tient, plus basse. La goutte jaune a séché sur le zeste. Le bois de l'étal redevient sec. Le citron mouillé a rejoint la tour, grain collé.</t>
+          <t>Le citron a failli tomber de la tour. On l'a rangé. Le stand est à nous. Vous avez offert le fruit. La tour tient, plus basse. La goutte jaune a séché sur le zeste. Le bois de l'étal redevient sec. Le citron mouillé a rejoint la tour, grain de cannelle collé.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le citron a failli tomber de la tour. On l'a rangé. Le stand est à nous. Vous avez offert le fruit. La tour tient, plus basse. La goutte jaune a séché sur le zeste. Le bois de l'étal redevient sec. Le citron mouillé a rejoint la tour, grain collé.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le citron a failli tomber de la tour. On l'a rangé. Le stand est à nous. Vous avez offert le fruit. La tour tient, plus basse. La goutte jaune a séché sur le zeste. Le bois de l'étal redevient sec. Le citron mouillé a rejoint la tour, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; collé.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le citron a failli tomber de la tour. On l'a rangé. Le stand est à nous. Vous avez offert le fruit. La tour tient, plus basse. La goutte jaune a séché sur le zeste. Le bois de l'étal redevient sec. Le citron mouillé a rejoint la tour, grain collé.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le citron a failli tomber de la tour. On l'a rangé. Le stand est à nous. Vous avez offert le fruit. La tour tient, plus basse. La goutte jaune a séché sur le zeste. Le bois de l'étal redevient sec. Le citron mouillé a rejoint la tour, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; collé.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -6823,7 +6826,7 @@
 maman|La tour tient, plus basse.
 narrateur|La goutte jaune a séché sur le zeste.
 narrateur|Le bois de l'étal redevient sec.
-narrateur|Le citron mouillé a rejoint la tour, grain collé.</t>
+narrateur|Le citron mouillé a rejoint la tour, grain de cannelle collé.</t>
         </is>
       </c>
       <c r="AX31" t="inlineStr">
@@ -6855,17 +6858,17 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Raphaël passe sous le store rouge. La toile chauffe les joues, d'une lumière rose. Les fraises sentent le sucre. La balance, le sac et la caisse restent là. Il saisit une fraise, trop vite. Pour toi, Mila ! Mila serre les poches. La fraise brille, seule, entre ses doigts. L'élan de Raphaël se casse. Elle n'a pas ouvert la main. Papa s'accroupit, au ras de la barquette. Une goutte rose glisse le long de la toile. Elle mouille le grain de cannelle, au bord. Il pique un peu, le grain. Tu le sens, sur le bois ?</t>
+          <t>Raphaël passe sous le store rouge. La toile chauffe les joues, d'une lumière rose. Les fraises sentent le sucre. La balance, le sac et la caisse restent là. Il saisit une fraise, trop vite. Pour toi, Mila ! Mila serre les poches. La fraise brille, seule, entre ses doigts. L'élan de Raphaël se casse. Elle n'a pas ouvert la main. Papa s'accroupit, au ras de la barquette. Une goutte rose glisse le long de la toile. Elle mouille le grain de cannelle, au bord. Il pique un peu, le grain. Tu le sens, sur le bois ? Une femme passe, le nez ailleurs.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël passe sous le &lt;emphasis level="moderate"&gt;store rouge&lt;/emphasis&gt;. La toile chauffe les joues, d'une lumière rose. Les fraises sentent le sucre. La balance, le sac et la caisse restent là. Il saisit une fraise, trop vite. Pour toi, Mila ! Mila serre les poches. La fraise brille, seule, entre ses doigts. L'élan de Raphaël se casse. Elle n'a pas ouvert la main. Papa s'accroupit, au ras de la barquette. Une goutte rose glisse le long de la toile. Elle mouille le grain de cannelle, au bord. Il pique un peu, le grain. Tu le sens, sur le bois ?&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël passe sous le &lt;emphasis level="moderate"&gt;store rouge&lt;/emphasis&gt;. La toile chauffe les joues, d'une lumière rose. Les fraises sentent le sucre. La balance, le sac et la caisse restent là. Il saisit une fraise, trop vite. Pour toi, Mila ! Mila serre les poches. La fraise brille, seule, entre ses doigts. L'élan de Raphaël se casse. Elle n'a pas ouvert la main. Papa s'accroupit, au ras de la barquette. Une goutte rose glisse le long de la toile. Elle mouille le grain de cannelle, au bord. Il pique un peu, le grain. Tu le sens, sur le bois ? Une femme passe, le nez ailleurs.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Raphaël passe sous le &lt;emphasis&gt;store rouge&lt;/emphasis&gt;. La toile chauffe les joues, d'une lumière rose. Les fraises sentent le sucre. La balance, le sac et la caisse restent là. Il saisit une fraise, trop vite. Pour toi, Mila ! Mila serre les poches. La fraise brille, seule, entre ses doigts. L'élan de Raphaël se casse. Elle n'a pas ouvert la main. Papa s'accroupit, au ras de la barquette. Une goutte rose glisse le long de la toile. Elle mouille le grain de cannelle, au bord. Il pique un peu, le grain. Tu le sens, sur le bois ? [pause]</t>
+          <t>Raphaël passe sous le &lt;emphasis&gt;store rouge&lt;/emphasis&gt;. La toile chauffe les joues, d'une lumière rose. Les fraises sentent le sucre. La balance, le sac et la caisse restent là. Il saisit une fraise, trop vite. Pour toi, Mila ! Mila serre les poches. La fraise brille, seule, entre ses doigts. L'élan de Raphaël se casse. Elle n'a pas ouvert la main. Papa s'accroupit, au ras de la barquette. Une goutte rose glisse le long de la toile. Elle mouille le grain de cannelle, au bord. Il pique un peu, le grain. Tu le sens, sur le bois ? Une femme passe, le nez ailleurs. [pause]</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -7013,7 +7016,8 @@
 narrateur|Une goutte rose glisse le long de la toile.
 narrateur|Elle mouille le grain de cannelle, au bord.
 enfant-m|Il pique un peu, le grain.
-maman|Tu le sens, sur le bois ?</t>
+maman|Tu le sens, sur le bois ?
+narrateur|Une femme passe, le nez ailleurs.</t>
         </is>
       </c>
       <c r="AX32" t="inlineStr">
@@ -8185,17 +8189,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Le jus a failli emporter le grain. Mila reste au bord, les yeux sur le rond. Tu as regardé le tic. Oui. L'aiguille s'est tue. La fraise a gardé sa place. La goutte rose a séché en rond mince. Un rond rose sèche, le grain au centre.</t>
+          <t>Le jus a failli emporter le grain. Mila reste au bord, les yeux sur le rond. Tu as regardé le tic. Oui. L'aiguille s'est tue. La fraise a gardé sa place. La goutte rose a séché en rond mince. Un rond rose sèche, le grain de cannelle au centre.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jus a failli emporter le grain. Mila reste au bord, les yeux sur le rond. Tu as regardé le tic. Oui. L'aiguille s'est tue. La fraise a gardé sa place. La goutte rose a séché en rond mince. Un rond rose sèche, le grain au centre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jus a failli emporter le grain. Mila reste au bord, les yeux sur le rond. Tu as regardé le tic. Oui. L'aiguille s'est tue. La fraise a gardé sa place. La goutte rose a séché en rond mince. Un rond rose sèche, le &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; au centre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jus a failli emporter le grain. Mila reste au bord, les yeux sur le rond. Tu as regardé le tic. Oui. L'aiguille s'est tue. La fraise a gardé sa place. La goutte rose a séché en rond mince. Un rond rose sèche, le grain au centre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jus a failli emporter le grain. Mila reste au bord, les yeux sur le rond. Tu as regardé le tic. Oui. L'aiguille s'est tue. La fraise a gardé sa place. La goutte rose a séché en rond mince. Un rond rose sèche, le &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; au centre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -8340,7 +8344,7 @@
 papa|L'aiguille s'est tue.
 maman|La fraise a gardé sa place.
 narrateur|La goutte rose a séché en rond mince.
-narrateur|Un rond rose sèche, le grain au centre.</t>
+narrateur|Un rond rose sèche, le grain de cannelle au centre.</t>
         </is>
       </c>
       <c r="AX39" t="inlineStr">
@@ -8372,17 +8376,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Plus tard. D'accord. Je te la garde. Raphaël garde la fraise sur le métal. Mila recule vers une odeur de pain, plus loin. La fraise garde sa place. Le grain de cannelle attend, à côté du fruit. Le plateau reste froid, pour elle.</t>
+          <t>Plus tard. D'accord. Je te la garde. Raphaël garde la fraise sur le métal. Mila recule vers une autre odeur, plus loin. La fraise garde sa place. Le grain de cannelle attend, à côté du fruit. Le plateau reste froid, pour elle.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus tard. D'accord. Je te la garde. Raphaël garde la fraise sur le métal. Mila recule vers une odeur de pain, plus loin. La fraise garde sa place. Le grain de cannelle attend, à côté du fruit. Le plateau reste froid, pour elle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus tard. D'accord. Je te la garde. Raphaël garde la fraise sur le métal. Mila recule vers une autre odeur, plus loin. La fraise garde sa place. Le grain de cannelle attend, à côté du fruit. Le plateau reste froid, pour elle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Plus tard. D'accord. Je te la garde. Raphaël garde la fraise sur le métal. Mila recule vers une odeur de pain, plus loin. La fraise garde sa place. Le grain de cannelle attend, à côté du fruit. Le plateau reste froid, pour elle. [pause]</t>
+          <t>Plus tard. D'accord. Je te la garde. Raphaël garde la fraise sur le métal. Mila recule vers une autre odeur, plus loin. La fraise garde sa place. Le grain de cannelle attend, à côté du fruit. Le plateau reste froid, pour elle. [pause]</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8520,7 +8524,7 @@
 enfant-m|D'accord.
 enfant-m|Je te la garde.
 narrateur|Raphaël garde la fraise sur le métal.
-narrateur|Mila recule vers une odeur de pain, plus loin.
+narrateur|Mila recule vers une autre odeur, plus loin.
 maman|La fraise garde sa place.
 narrateur|Le grain de cannelle attend, à côté du fruit.
 papa|Le plateau reste froid, pour elle.</t>
@@ -8555,17 +8559,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Mila revient, une miette de pain au coin des lèvres. Maintenant ? Oui. Elle s'approche de la balance. Vous avez pris le temps. La fraise l'attendait. La goutte rose n'est plus qu'un halo. La fraise garde sa place, grain à côté.</t>
+          <t>Mila revient, une miette sucrée au coin des lèvres. Maintenant ? Oui. Elle s'approche de la balance. Vous avez pris le temps. La fraise l'attendait. La goutte rose n'est plus qu'un halo. La fraise garde sa place, grain de cannelle à côté.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, une miette de pain au coin des lèvres. Maintenant ? Oui. Elle s'approche de la balance. Vous avez pris le temps. La fraise l'attendait. La goutte rose n'est plus qu'un halo. La fraise garde sa place, grain à côté.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, une miette sucrée au coin des lèvres. Maintenant ? Oui. Elle s'approche de la balance. Vous avez pris le temps. La fraise l'attendait. La goutte rose n'est plus qu'un halo. La fraise garde sa place, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; à côté.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, une miette de pain au coin des lèvres. Maintenant ? Oui. Elle s'approche de la balance. Vous avez pris le temps. La fraise l'attendait. La goutte rose n'est plus qu'un halo. La fraise garde sa place, grain à côté.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, une miette sucrée au coin des lèvres. Maintenant ? Oui. Elle s'approche de la balance. Vous avez pris le temps. La fraise l'attendait. La goutte rose n'est plus qu'un halo. La fraise garde sa place, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; à côté.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8703,14 +8707,14 @@
       </c>
       <c r="AW41" t="inlineStr">
         <is>
-          <t>narrateur|Mila revient, une miette de pain au coin des lèvres.
+          <t>narrateur|Mila revient, une miette sucrée au coin des lèvres.
 enfant-f|Maintenant ?
 enfant-m|Oui.
 narrateur|Elle s'approche de la balance.
 papa|Vous avez pris le temps.
 maman|La fraise l'attendait.
 narrateur|La goutte rose n'est plus qu'un halo.
-narrateur|La fraise garde sa place, grain à côté.</t>
+narrateur|La fraise garde sa place, grain de cannelle à côté.</t>
         </is>
       </c>
       <c r="AX41" t="inlineStr">
@@ -8925,17 +8929,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>La fraise a failli glisser dans le jus. On l'a pesée. Le stand est à nous. Vous avez offert le fruit. Deux doigts ont gardé le grain. La goutte rose a quitté le métal. Le bois de l'étal redevient sec. L'aiguille s'est tue, grain sous deux doigts.</t>
+          <t>La fraise a failli glisser dans le jus. On l'a pesée. Le stand est à nous. Vous avez offert le fruit. Deux doigts ont gardé le grain. La goutte rose a quitté le métal. Le bois de l'étal redevient sec. L'aiguille s'est tue, grain de cannelle sous deux doigts.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La fraise a failli glisser dans le jus. On l'a pesée. Le stand est à nous. Vous avez offert le fruit. Deux doigts ont gardé le grain. La goutte rose a quitté le métal. Le bois de l'étal redevient sec. L'aiguille s'est tue, grain sous deux doigts.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La fraise a failli glisser dans le jus. On l'a pesée. Le stand est à nous. Vous avez offert le fruit. Deux doigts ont gardé le grain. La goutte rose a quitté le métal. Le bois de l'étal redevient sec. L'aiguille s'est tue, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; sous deux doigts.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La fraise a failli glisser dans le jus. On l'a pesée. Le stand est à nous. Vous avez offert le fruit. Deux doigts ont gardé le grain. La goutte rose a quitté le métal. Le bois de l'étal redevient sec. L'aiguille s'est tue, grain sous deux doigts.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La fraise a failli glisser dans le jus. On l'a pesée. Le stand est à nous. Vous avez offert le fruit. Deux doigts ont gardé le grain. La goutte rose a quitté le métal. Le bois de l'étal redevient sec. L'aiguille s'est tue, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; sous deux doigts.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -9080,7 +9084,7 @@
 maman|Deux doigts ont gardé le grain.
 narrateur|La goutte rose a quitté le métal.
 narrateur|Le bois de l'étal redevient sec.
-narrateur|L'aiguille s'est tue, grain sous deux doigts.</t>
+narrateur|L'aiguille s'est tue, grain de cannelle sous deux doigts.</t>
         </is>
       </c>
       <c r="AX43" t="inlineStr">
@@ -9685,17 +9689,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Le sac a failli avaler le grain. Mila reste au bord, le nez dans le pli. Tu as regardé le pli. Oui. Le papier est resté ouvert. Le sucre habite le brun. La goutte rose a séché dans le pli. Le sac sent le sucre, grain coincé dans le pli.</t>
+          <t>Le sac a failli avaler le grain. Mila reste au bord, le nez dans le pli. Tu as regardé le pli. Oui. Le papier est resté ouvert. Le sucre habite le brun. La goutte rose a séché dans le pli. Le sac sent le sucre, grain de cannelle coincé dans le pli.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le sac a failli avaler le grain. Mila reste au bord, le nez dans le pli. Tu as regardé le pli. Oui. Le papier est resté ouvert. Le sucre habite le brun. La goutte rose a séché dans le pli. Le sac sent le sucre, grain coincé dans le pli.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le sac a failli avaler le grain. Mila reste au bord, le nez dans le pli. Tu as regardé le pli. Oui. Le papier est resté ouvert. Le sucre habite le brun. La goutte rose a séché dans le pli. Le sac sent le sucre, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; coincé dans le pli.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le sac a failli avaler le grain. Mila reste au bord, le nez dans le pli. Tu as regardé le pli. Oui. Le papier est resté ouvert. Le sucre habite le brun. La goutte rose a séché dans le pli. Le sac sent le sucre, grain coincé dans le pli.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le sac a failli avaler le grain. Mila reste au bord, le nez dans le pli. Tu as regardé le pli. Oui. Le papier est resté ouvert. Le sucre habite le brun. La goutte rose a séché dans le pli. Le sac sent le sucre, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; coincé dans le pli.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9840,7 +9844,7 @@
 papa|Le papier est resté ouvert.
 maman|Le sucre habite le brun.
 narrateur|La goutte rose a séché dans le pli.
-narrateur|Le sac sent le sucre, grain coincé dans le pli.</t>
+narrateur|Le sac sent le sucre, grain de cannelle coincé dans le pli.</t>
         </is>
       </c>
       <c r="AX47" t="inlineStr">
@@ -10055,17 +10059,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Mila revient, les doigts un peu collants. Maintenant ? Oui, le sac est là. Elle s'approche du papier. Vous avez pris le temps. La barquette l'attendait. La goutte rose a quitté le col. La barquette attend, grain sur le papier.</t>
+          <t>Mila revient, les doigts un peu collants. Maintenant ? Oui, le sac est là. Elle s'approche du papier. Vous avez pris le temps. La barquette l'attendait. La goutte rose a quitté le col. La barquette attend, grain de cannelle sur le papier.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, les doigts un peu collants. Maintenant ? Oui, le sac est là. Elle s'approche du papier. Vous avez pris le temps. La barquette l'attendait. La goutte rose a quitté le col. La barquette attend, grain sur le papier.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, les doigts un peu collants. Maintenant ? Oui, le sac est là. Elle s'approche du papier. Vous avez pris le temps. La barquette l'attendait. La goutte rose a quitté le col. La barquette attend, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; sur le papier.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, les doigts un peu collants. Maintenant ? Oui, le sac est là. Elle s'approche du papier. Vous avez pris le temps. La barquette l'attendait. La goutte rose a quitté le col. La barquette attend, grain sur le papier.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, les doigts un peu collants. Maintenant ? Oui, le sac est là. Elle s'approche du papier. Vous avez pris le temps. La barquette l'attendait. La goutte rose a quitté le col. La barquette attend, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; sur le papier.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10210,7 +10214,7 @@
 papa|Vous avez pris le temps.
 maman|La barquette l'attendait.
 narrateur|La goutte rose a quitté le col.
-narrateur|La barquette attend, grain sur le papier.</t>
+narrateur|La barquette attend, grain de cannelle sur le papier.</t>
         </is>
       </c>
       <c r="AX49" t="inlineStr">
@@ -10425,17 +10429,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Les fraises ont failli s'écraser au fond. On l'a porté. Le stand est à nous. Vous avez offert le fruit. Le sac froisse, porté à deux. La goutte rose a séché au fond. Le bois de l'étal redevient sec. Le sac froisse, porté à deux, grain dedans.</t>
+          <t>Les fraises ont failli s'écraser au fond. On l'a porté. Le stand est à nous. Vous avez offert le fruit. Le sac froisse, porté à deux. La goutte rose a séché au fond. Le bois de l'étal redevient sec. Le sac froisse, porté à deux, grain de cannelle dedans.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les fraises ont failli s'écraser au fond. On l'a porté. Le stand est à nous. Vous avez offert le fruit. Le sac froisse, porté à deux. La goutte rose a séché au fond. Le bois de l'étal redevient sec. Le sac froisse, porté à deux, grain dedans.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les fraises ont failli s'écraser au fond. On l'a porté. Le stand est à nous. Vous avez offert le fruit. Le sac froisse, porté à deux. La goutte rose a séché au fond. Le bois de l'étal redevient sec. Le sac froisse, porté à deux, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; dedans.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les fraises ont failli s'écraser au fond. On l'a porté. Le stand est à nous. Vous avez offert le fruit. Le sac froisse, porté à deux. La goutte rose a séché au fond. Le bois de l'étal redevient sec. Le sac froisse, porté à deux, grain dedans.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les fraises ont failli s'écraser au fond. On l'a porté. Le stand est à nous. Vous avez offert le fruit. Le sac froisse, porté à deux. La goutte rose a séché au fond. Le bois de l'étal redevient sec. Le sac froisse, porté à deux, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; dedans.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -10580,7 +10584,7 @@
 maman|Le sac froisse, porté à deux.
 narrateur|La goutte rose a séché au fond.
 narrateur|Le bois de l'étal redevient sec.
-narrateur|Le sac froisse, porté à deux, grain dedans.</t>
+narrateur|Le sac froisse, porté à deux, grain de cannelle dedans.</t>
         </is>
       </c>
       <c r="AX51" t="inlineStr">
@@ -11185,17 +11189,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>La rangée a failli tout emporter. Mila reste au bord, les yeux sur le bois. Tu as regardé la place. Oui. Les fraises sont alignées, sous le rouge. Le bois a gardé un creux. La goutte rose a séché sur la planche. Les fraises sont alignées, grain sur le bois rouge.</t>
+          <t>La rangée a failli tout emporter. Mila reste au bord, les yeux sur le bois. Tu as regardé la place. Oui. Les fraises sont alignées, sous le rouge. Le bois a gardé un creux. La goutte rose a séché sur la planche. Les fraises sont alignées, grain de cannelle sur le bois rouge.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La rangée a failli tout emporter. Mila reste au bord, les yeux sur le bois. Tu as regardé la place. Oui. Les fraises sont alignées, sous le rouge. Le bois a gardé un creux. La goutte rose a séché sur la planche. Les fraises sont alignées, grain sur le bois rouge.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La rangée a failli tout emporter. Mila reste au bord, les yeux sur le bois. Tu as regardé la place. Oui. Les fraises sont alignées, sous le rouge. Le bois a gardé un creux. La goutte rose a séché sur la planche. Les fraises sont alignées, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; sur le bois rouge.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La rangée a failli tout emporter. Mila reste au bord, les yeux sur le bois. Tu as regardé la place. Oui. Les fraises sont alignées, sous le rouge. Le bois a gardé un creux. La goutte rose a séché sur la planche. Les fraises sont alignées, grain sur le bois rouge.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La rangée a failli tout emporter. Mila reste au bord, les yeux sur le bois. Tu as regardé la place. Oui. Les fraises sont alignées, sous le rouge. Le bois a gardé un creux. La goutte rose a séché sur la planche. Les fraises sont alignées, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; sur le bois rouge.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11340,7 +11344,7 @@
 papa|Les fraises sont alignées, sous le rouge.
 maman|Le bois a gardé un creux.
 narrateur|La goutte rose a séché sur la planche.
-narrateur|Les fraises sont alignées, grain sur le bois rouge.</t>
+narrateur|Les fraises sont alignées, grain de cannelle sur le bois rouge.</t>
         </is>
       </c>
       <c r="AX55" t="inlineStr">
@@ -11555,17 +11559,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Mila revient, une main hors de la poche. Maintenant ? Oui, ta place est là. Elle s'approche de la caisse. Vous avez pris le temps. La place rose l'attendait. La goutte rose a quitté le bord. Une place rose reste, grain au creux.</t>
+          <t>Mila revient, une main hors de la poche. Maintenant ? Oui, ta place est là. Elle s'approche de la caisse. Vous avez pris le temps. La place rose l'attendait. La goutte rose a quitté le bord. Une place rose reste, grain de cannelle au creux.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, une main hors de la poche. Maintenant ? Oui, ta place est là. Elle s'approche de la caisse. Vous avez pris le temps. La place rose l'attendait. La goutte rose a quitté le bord. Une place rose reste, grain au creux.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, une main hors de la poche. Maintenant ? Oui, ta place est là. Elle s'approche de la caisse. Vous avez pris le temps. La place rose l'attendait. La goutte rose a quitté le bord. Une place rose reste, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; au creux.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, une main hors de la poche. Maintenant ? Oui, ta place est là. Elle s'approche de la caisse. Vous avez pris le temps. La place rose l'attendait. La goutte rose a quitté le bord. Une place rose reste, grain au creux.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, une main hors de la poche. Maintenant ? Oui, ta place est là. Elle s'approche de la caisse. Vous avez pris le temps. La place rose l'attendait. La goutte rose a quitté le bord. Une place rose reste, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; au creux.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11710,7 +11714,7 @@
 papa|Vous avez pris le temps.
 maman|La place rose l'attendait.
 narrateur|La goutte rose a quitté le bord.
-narrateur|Une place rose reste, grain au creux.</t>
+narrateur|Une place rose reste, grain de cannelle au creux.</t>
         </is>
       </c>
       <c r="AX57" t="inlineStr">
@@ -11925,17 +11929,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>La fraise a failli rouler hors de la caisse. On l'a rangée. Le stand est à nous. Vous avez offert le fruit. La rangée tient, fermée. La goutte rose a séché sur le fruit. Le bois de l'étal redevient sec. La fraise rattrapée ne roule plus, grain dessus.</t>
+          <t>La fraise a failli rouler hors de la caisse. On l'a rangée. Le stand est à nous. Vous avez offert le fruit. La rangée tient, fermée. La goutte rose a séché sur le fruit. Le bois de l'étal redevient sec. La fraise rattrapée ne roule plus, grain de cannelle dessus.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La fraise a failli rouler hors de la caisse. On l'a rangée. Le stand est à nous. Vous avez offert le fruit. La rangée tient, fermée. La goutte rose a séché sur le fruit. Le bois de l'étal redevient sec. La fraise rattrapée ne roule plus, grain dessus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La fraise a failli rouler hors de la caisse. On l'a rangée. Le stand est à nous. Vous avez offert le fruit. La rangée tient, fermée. La goutte rose a séché sur le fruit. Le bois de l'étal redevient sec. La fraise rattrapée ne roule plus, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; dessus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La fraise a failli rouler hors de la caisse. On l'a rangée. Le stand est à nous. Vous avez offert le fruit. La rangée tient, fermée. La goutte rose a séché sur le fruit. Le bois de l'étal redevient sec. La fraise rattrapée ne roule plus, grain dessus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La fraise a failli rouler hors de la caisse. On l'a rangée. Le stand est à nous. Vous avez offert le fruit. La rangée tient, fermée. La goutte rose a séché sur le fruit. Le bois de l'étal redevient sec. La fraise rattrapée ne roule plus, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; dessus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -12080,7 +12084,7 @@
 maman|La rangée tient, fermée.
 narrateur|La goutte rose a séché sur le fruit.
 narrateur|Le bois de l'étal redevient sec.
-narrateur|La fraise rattrapée ne roule plus, grain dessus.</t>
+narrateur|La fraise rattrapée ne roule plus, grain de cannelle dessus.</t>
         </is>
       </c>
       <c r="AX59" t="inlineStr">
@@ -12112,17 +12116,17 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Raphaël s'abrite sous le store vert. La toile pose des taches vertes sur les poires. Elles sont lourdes. La balance, le sac et la caisse restent là. Il soulève une poire, trop vite. Tiens, Mila ! Mila baisse les yeux. La poire pèse, seule, contre son ventre. Dans sa poitrine, ça serre, fort. Elle n'a pas levé les mains. Maman s'accroupit, à hauteur de l'étal. Une goutte verte pend, trop ronde. Elle tombe près du grain de cannelle. Le grain a un point d'eau. Tu le vois, collé au bois ?</t>
+          <t>Raphaël s'abrite sous le store vert. La toile pose des taches vertes sur les poires. Elles sont lourdes. La balance, le sac et la caisse restent là. Il soulève une poire, trop vite. Tiens, Mila ! Mila baisse les yeux. La poire pèse, seule, contre son ventre. Dans sa poitrine, ça serre, fort. Elle n'a pas levé les mains. Maman s'accroupit, à hauteur de l'étal. Une goutte verte pend, trop ronde. Elle tombe près du grain de cannelle. Le grain a un point d'eau. Tu le vois, collé au bois ? Un homme passe, sans regarder l'étal.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël s'abrite sous le &lt;emphasis level="moderate"&gt;store vert&lt;/emphasis&gt;. La toile pose des taches vertes sur les poires. Elles sont lourdes. La balance, le sac et la caisse restent là. Il soulève une poire, trop vite. Tiens, Mila ! Mila baisse les yeux. La poire pèse, seule, contre son ventre. Dans sa poitrine, ça serre, fort. Elle n'a pas levé les mains. Maman s'accroupit, à hauteur de l'étal. Une goutte verte pend, trop ronde. Elle tombe près du grain de cannelle. Le grain a un point d'eau. Tu le vois, collé au bois ?&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël s'abrite sous le &lt;emphasis level="moderate"&gt;store vert&lt;/emphasis&gt;. La toile pose des taches vertes sur les poires. Elles sont lourdes. La balance, le sac et la caisse restent là. Il soulève une poire, trop vite. Tiens, Mila ! Mila baisse les yeux. La poire pèse, seule, contre son ventre. Dans sa poitrine, ça serre, fort. Elle n'a pas levé les mains. Maman s'accroupit, à hauteur de l'étal. Une goutte verte pend, trop ronde. Elle tombe près du grain de cannelle. Le grain a un point d'eau. Tu le vois, collé au bois ? Un homme passe, sans regarder l'étal.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Raphaël s'abrite sous le &lt;emphasis&gt;store vert&lt;/emphasis&gt;. La toile pose des taches vertes sur les poires. Elles sont lourdes. La balance, le sac et la caisse restent là. Il soulève une poire, trop vite. Tiens, Mila ! Mila baisse les yeux. La poire pèse, seule, contre son ventre. Dans sa poitrine, ça serre, fort. Elle n'a pas levé les mains. Maman s'accroupit, à hauteur de l'étal. Une goutte verte pend, trop ronde. Elle tombe près du grain de cannelle. Le grain a un point d'eau. Tu le vois, collé au bois ? [pause]</t>
+          <t>Raphaël s'abrite sous le &lt;emphasis&gt;store vert&lt;/emphasis&gt;. La toile pose des taches vertes sur les poires. Elles sont lourdes. La balance, le sac et la caisse restent là. Il soulève une poire, trop vite. Tiens, Mila ! Mila baisse les yeux. La poire pèse, seule, contre son ventre. Dans sa poitrine, ça serre, fort. Elle n'a pas levé les mains. Maman s'accroupit, à hauteur de l'étal. Une goutte verte pend, trop ronde. Elle tombe près du grain de cannelle. Le grain a un point d'eau. Tu le vois, collé au bois ? Un homme passe, sans regarder l'étal. [pause]</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -12270,7 +12274,8 @@
 narrateur|Une goutte verte pend, trop ronde.
 narrateur|Elle tombe près du grain de cannelle.
 enfant-m|Le grain a un point d'eau.
-papa|Tu le vois, collé au bois ?</t>
+papa|Tu le vois, collé au bois ?
+narrateur|Un homme passe, sans regarder l'étal.</t>
         </is>
       </c>
       <c r="AX60" t="inlineStr">
@@ -13442,17 +13447,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Le plateau a failli tout verser. Mila reste au bord, les yeux sur le chiffre. Tu as regardé le chiffre. Oui. Le chiffre noir reste grand. La poire a gardé sa place. La goutte verte a séché en virgule mince. Le chiffre noir reste grand, grain contre le plateau.</t>
+          <t>Le plateau a failli tout verser. Mila reste au bord, les yeux sur le chiffre. Tu as regardé le chiffre. Oui. Le chiffre noir reste grand. La poire a gardé sa place. La goutte verte a séché en trait d'eau. Le chiffre noir reste grand, grain de cannelle contre le plateau.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le plateau a failli tout verser. Mila reste au bord, les yeux sur le chiffre. Tu as regardé le chiffre. Oui. Le chiffre noir reste grand. La poire a gardé sa place. La goutte verte a séché en virgule mince. Le chiffre noir reste grand, grain contre le plateau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le plateau a failli tout verser. Mila reste au bord, les yeux sur le chiffre. Tu as regardé le chiffre. Oui. Le chiffre noir reste grand. La poire a gardé sa place. La goutte verte a séché en trait d'eau. Le chiffre noir reste grand, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; contre le plateau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le plateau a failli tout verser. Mila reste au bord, les yeux sur le chiffre. Tu as regardé le chiffre. Oui. Le chiffre noir reste grand. La poire a gardé sa place. La goutte verte a séché en virgule mince. Le chiffre noir reste grand, grain contre le plateau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le plateau a failli tout verser. Mila reste au bord, les yeux sur le chiffre. Tu as regardé le chiffre. Oui. Le chiffre noir reste grand. La poire a gardé sa place. La goutte verte a séché en trait d'eau. Le chiffre noir reste grand, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; contre le plateau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -13596,8 +13601,8 @@
 enfant-f|Oui.
 papa|Le chiffre noir reste grand.
 maman|La poire a gardé sa place.
-narrateur|La goutte verte a séché en virgule mince.
-narrateur|Le chiffre noir reste grand, grain contre le plateau.</t>
+narrateur|La goutte verte a séché en trait d'eau.
+narrateur|Le chiffre noir reste grand, grain de cannelle contre le plateau.</t>
         </is>
       </c>
       <c r="AX67" t="inlineStr">
@@ -13812,17 +13817,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Mila revient, une feuille collée à la chaussure. Maintenant ? Oui. Elle s'approche de la balance. Vous avez pris le temps. La poire l'attendait. La goutte verte n'est plus qu'un point. La poire pèse, grain à l'abri sous le fruit.</t>
+          <t>Mila revient, une feuille collée à la chaussure. Maintenant ? Oui. Elle s'approche de la balance. Vous avez pris le temps. La poire l'attendait. La goutte verte n'est plus qu'un point. La poire pèse, grain de cannelle à l'abri sous le fruit.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, une feuille collée à la chaussure. Maintenant ? Oui. Elle s'approche de la balance. Vous avez pris le temps. La poire l'attendait. La goutte verte n'est plus qu'un point. La poire pèse, grain à l'abri sous le fruit.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, une feuille collée à la chaussure. Maintenant ? Oui. Elle s'approche de la balance. Vous avez pris le temps. La poire l'attendait. La goutte verte n'est plus qu'un point. La poire pèse, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; à l'abri sous le fruit.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, une feuille collée à la chaussure. Maintenant ? Oui. Elle s'approche de la balance. Vous avez pris le temps. La poire l'attendait. La goutte verte n'est plus qu'un point. La poire pèse, grain à l'abri sous le fruit.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, une feuille collée à la chaussure. Maintenant ? Oui. Elle s'approche de la balance. Vous avez pris le temps. La poire l'attendait. La goutte verte n'est plus qu'un point. La poire pèse, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; à l'abri sous le fruit.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -13967,7 +13972,7 @@
 papa|Vous avez pris le temps.
 maman|La poire l'attendait.
 narrateur|La goutte verte n'est plus qu'un point.
-narrateur|La poire pèse, grain à l'abri sous le fruit.</t>
+narrateur|La poire pèse, grain de cannelle à l'abri sous le fruit.</t>
         </is>
       </c>
       <c r="AX69" t="inlineStr">
@@ -14182,17 +14187,17 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>La poire a failli faire pencher tout le plateau. On l'a pesée. Le stand est à nous. Vous avez offert le fruit. Le plateau s'est calmé, entre eux. La goutte verte a quitté la peau. Le bois de l'étal redevient sec. Le plateau s'est calmé, grain entre eux.</t>
+          <t>La poire a failli faire pencher tout le plateau. On l'a pesée. Le stand est à nous. Vous avez offert le fruit. Le plateau s'est calmé, entre eux. La goutte verte a quitté la peau. Le bois de l'étal redevient sec. Le plateau s'est calmé, grain de cannelle entre eux.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La poire a failli faire pencher tout le plateau. On l'a pesée. Le stand est à nous. Vous avez offert le fruit. Le plateau s'est calmé, entre eux. La goutte verte a quitté la peau. Le bois de l'étal redevient sec. Le plateau s'est calmé, grain entre eux.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La poire a failli faire pencher tout le plateau. On l'a pesée. Le stand est à nous. Vous avez offert le fruit. Le plateau s'est calmé, entre eux. La goutte verte a quitté la peau. Le bois de l'étal redevient sec. Le plateau s'est calmé, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; entre eux.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La poire a failli faire pencher tout le plateau. On l'a pesée. Le stand est à nous. Vous avez offert le fruit. Le plateau s'est calmé, entre eux. La goutte verte a quitté la peau. Le bois de l'étal redevient sec. Le plateau s'est calmé, grain entre eux.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La poire a failli faire pencher tout le plateau. On l'a pesée. Le stand est à nous. Vous avez offert le fruit. Le plateau s'est calmé, entre eux. La goutte verte a quitté la peau. Le bois de l'étal redevient sec. Le plateau s'est calmé, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; entre eux.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -14337,7 +14342,7 @@
 maman|Le plateau s'est calmé, entre eux.
 narrateur|La goutte verte a quitté la peau.
 narrateur|Le bois de l'étal redevient sec.
-narrateur|Le plateau s'est calmé, grain entre eux.</t>
+narrateur|Le plateau s'est calmé, grain de cannelle entre eux.</t>
         </is>
       </c>
       <c r="AX71" t="inlineStr">
@@ -14942,17 +14947,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Le sac a failli se déchirer jusqu'au fond. Mila reste au bord, les yeux sur la tache. Tu as regardé le col. Oui. Le sac a pris la forme de la poire. Le sucré habite le brun. La goutte verte a séché au col. Le sac a pris la forme de la poire, grain au col.</t>
+          <t>Le sac a failli se déchirer jusqu'au fond. Mila reste au bord, les yeux sur la tache. Tu as regardé le col. Oui. Le sac a pris la forme de la poire. Le sucré habite le brun. La goutte verte a séché au col. Le sac a pris la forme de la poire, grain de cannelle au col.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le sac a failli se déchirer jusqu'au fond. Mila reste au bord, les yeux sur la tache. Tu as regardé le col. Oui. Le sac a pris la forme de la poire. Le sucré habite le brun. La goutte verte a séché au col. Le sac a pris la forme de la poire, grain au col.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le sac a failli se déchirer jusqu'au fond. Mila reste au bord, les yeux sur la tache. Tu as regardé le col. Oui. Le sac a pris la forme de la poire. Le sucré habite le brun. La goutte verte a séché au col. Le sac a pris la forme de la poire, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; au col.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le sac a failli se déchirer jusqu'au fond. Mila reste au bord, les yeux sur la tache. Tu as regardé le col. Oui. Le sac a pris la forme de la poire. Le sucré habite le brun. La goutte verte a séché au col. Le sac a pris la forme de la poire, grain au col.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le sac a failli se déchirer jusqu'au fond. Mila reste au bord, les yeux sur la tache. Tu as regardé le col. Oui. Le sac a pris la forme de la poire. Le sucré habite le brun. La goutte verte a séché au col. Le sac a pris la forme de la poire, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; au col.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -15097,7 +15102,7 @@
 papa|Le sac a pris la forme de la poire.
 maman|Le sucré habite le brun.
 narrateur|La goutte verte a séché au col.
-narrateur|Le sac a pris la forme de la poire, grain au col.</t>
+narrateur|Le sac a pris la forme de la poire, grain de cannelle au col.</t>
         </is>
       </c>
       <c r="AX75" t="inlineStr">
@@ -15312,17 +15317,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Mila revient, les mains hors des poches. Maintenant ? Oui, le sac est là. Elle s'approche du papier. Vous avez pris le temps. Le papier l'attendait, lourd. La goutte verte a quitté le brun. Le papier attend, grain brun sur le brun.</t>
+          <t>Mila revient, les mains hors des poches. Maintenant ? Oui, le sac est là. Elle s'approche du papier. Vous avez pris le temps. Le papier l'attendait, lourd. La goutte verte a quitté le brun. Le papier attend, grain de cannelle brun sur le brun.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, les mains hors des poches. Maintenant ? Oui, le sac est là. Elle s'approche du papier. Vous avez pris le temps. Le papier l'attendait, lourd. La goutte verte a quitté le brun. Le papier attend, grain brun sur le brun.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, les mains hors des poches. Maintenant ? Oui, le sac est là. Elle s'approche du papier. Vous avez pris le temps. Le papier l'attendait, lourd. La goutte verte a quitté le brun. Le papier attend, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; brun sur le brun.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, les mains hors des poches. Maintenant ? Oui, le sac est là. Elle s'approche du papier. Vous avez pris le temps. Le papier l'attendait, lourd. La goutte verte a quitté le brun. Le papier attend, grain brun sur le brun.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, les mains hors des poches. Maintenant ? Oui, le sac est là. Elle s'approche du papier. Vous avez pris le temps. Le papier l'attendait, lourd. La goutte verte a quitté le brun. Le papier attend, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; brun sur le brun.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -15467,7 +15472,7 @@
 papa|Vous avez pris le temps.
 maman|Le papier l'attendait, lourd.
 narrateur|La goutte verte a quitté le brun.
-narrateur|Le papier attend, grain brun sur le brun.</t>
+narrateur|Le papier attend, grain de cannelle brun sur le brun.</t>
         </is>
       </c>
       <c r="AX77" t="inlineStr">
@@ -15682,17 +15687,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>La poire a failli fendre le sac. On l'a portée. Le stand est à nous. Vous avez offert le fruit. Le sac penche, puis tient. La goutte verte a séché au fond. Le bois de l'étal redevient sec. Le sac penche, puis tient, grain au fond.</t>
+          <t>La poire a failli fendre le sac. On l'a portée. Le stand est à nous. Vous avez offert le fruit. Le sac penche, puis tient. La goutte verte a séché au fond. Le bois de l'étal redevient sec. Le sac penche, puis tient, grain de cannelle au fond.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La poire a failli fendre le sac. On l'a portée. Le stand est à nous. Vous avez offert le fruit. Le sac penche, puis tient. La goutte verte a séché au fond. Le bois de l'étal redevient sec. Le sac penche, puis tient, grain au fond.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La poire a failli fendre le sac. On l'a portée. Le stand est à nous. Vous avez offert le fruit. Le sac penche, puis tient. La goutte verte a séché au fond. Le bois de l'étal redevient sec. Le sac penche, puis tient, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; au fond.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La poire a failli fendre le sac. On l'a portée. Le stand est à nous. Vous avez offert le fruit. Le sac penche, puis tient. La goutte verte a séché au fond. Le bois de l'étal redevient sec. Le sac penche, puis tient, grain au fond.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La poire a failli fendre le sac. On l'a portée. Le stand est à nous. Vous avez offert le fruit. Le sac penche, puis tient. La goutte verte a séché au fond. Le bois de l'étal redevient sec. Le sac penche, puis tient, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; au fond.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -15837,7 +15842,7 @@
 maman|Le sac penche, puis tient.
 narrateur|La goutte verte a séché au fond.
 narrateur|Le bois de l'étal redevient sec.
-narrateur|Le sac penche, puis tient, grain au fond.</t>
+narrateur|Le sac penche, puis tient, grain de cannelle au fond.</t>
         </is>
       </c>
       <c r="AX79" t="inlineStr">
@@ -16442,17 +16447,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>La tour a failli cacher toutes les poires. Mila reste au bord, les yeux sur le bas. Tu as regardé en bas. Oui. Les poires d'en bas restent à hauteur. La petite a gardé sa joue. La goutte verte a séché sur la planche. Les poires d'en bas restent à hauteur, grain sur la plus petite.</t>
+          <t>La tour a failli cacher toutes les poires. Mila reste au bord, les yeux sur le bas. Tu as regardé en bas. Oui. Les poires d'en bas restent à hauteur. La petite a gardé sa joue. La goutte verte a séché sur la planche. Les poires d'en bas restent à hauteur, grain de cannelle sur la plus petite.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La tour a failli cacher toutes les poires. Mila reste au bord, les yeux sur le bas. Tu as regardé en bas. Oui. Les poires d'en bas restent à hauteur. La petite a gardé sa joue. La goutte verte a séché sur la planche. Les poires d'en bas restent à hauteur, grain sur la plus petite.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La tour a failli cacher toutes les poires. Mila reste au bord, les yeux sur le bas. Tu as regardé en bas. Oui. Les poires d'en bas restent à hauteur. La petite a gardé sa joue. La goutte verte a séché sur la planche. Les poires d'en bas restent à hauteur, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; sur la plus petite.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La tour a failli cacher toutes les poires. Mila reste au bord, les yeux sur le bas. Tu as regardé en bas. Oui. Les poires d'en bas restent à hauteur. La petite a gardé sa joue. La goutte verte a séché sur la planche. Les poires d'en bas restent à hauteur, grain sur la plus petite.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La tour a failli cacher toutes les poires. Mila reste au bord, les yeux sur le bas. Tu as regardé en bas. Oui. Les poires d'en bas restent à hauteur. La petite a gardé sa joue. La goutte verte a séché sur la planche. Les poires d'en bas restent à hauteur, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; sur la plus petite.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16597,7 +16602,7 @@
 papa|Les poires d'en bas restent à hauteur.
 maman|La petite a gardé sa joue.
 narrateur|La goutte verte a séché sur la planche.
-narrateur|Les poires d'en bas restent à hauteur, grain sur la plus petite.</t>
+narrateur|Les poires d'en bas restent à hauteur, grain de cannelle sur la plus petite.</t>
         </is>
       </c>
       <c r="AX83" t="inlineStr">
@@ -16812,17 +16817,17 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Mila revient, une main sur le bord de l'étal. Maintenant ? Oui, ta poire est là. Elle s'approche de la caisse. Vous avez pris le temps. La petite l'attendait. La goutte verte a quitté le bord. Une poire du bas attend, grain sur sa joue.</t>
+          <t>Mila revient, une main sur le bord de l'étal. Maintenant ? Oui, ta poire est là. Elle s'approche de la caisse. Vous avez pris le temps. La petite l'attendait. La goutte verte a quitté le bord. Une poire du bas attend, grain de cannelle sur sa joue.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, une main sur le bord de l'étal. Maintenant ? Oui, ta poire est là. Elle s'approche de la caisse. Vous avez pris le temps. La petite l'attendait. La goutte verte a quitté le bord. Une poire du bas attend, grain sur sa joue.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila revient, une main sur le bord de l'étal. Maintenant ? Oui, ta poire est là. Elle s'approche de la caisse. Vous avez pris le temps. La petite l'attendait. La goutte verte a quitté le bord. Une poire du bas attend, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; sur sa joue.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, une main sur le bord de l'étal. Maintenant ? Oui, ta poire est là. Elle s'approche de la caisse. Vous avez pris le temps. La petite l'attendait. La goutte verte a quitté le bord. Une poire du bas attend, grain sur sa joue.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila revient, une main sur le bord de l'étal. Maintenant ? Oui, ta poire est là. Elle s'approche de la caisse. Vous avez pris le temps. La petite l'attendait. La goutte verte a quitté le bord. Une poire du bas attend, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; sur sa joue.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -16967,7 +16972,7 @@
 papa|Vous avez pris le temps.
 maman|La petite l'attendait.
 narrateur|La goutte verte a quitté le bord.
-narrateur|Une poire du bas attend, grain sur sa joue.</t>
+narrateur|Une poire du bas attend, grain de cannelle sur sa joue.</t>
         </is>
       </c>
       <c r="AX85" t="inlineStr">
@@ -17182,17 +17187,17 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>La poire d'en haut a failli tout cacher. On l'a prise, en bas. Le stand est à nous. Vous avez offert le fruit. La poire d'en bas a trouvé sa place. La goutte verte a séché sur sa joue. Le bois de l'étal redevient sec. La poire d'en bas a trouvé sa place, grain voyageur.</t>
+          <t>La poire d'en haut a failli tout cacher. On l'a prise, en bas. Le stand est à nous. Vous avez offert le fruit. La poire d'en bas a trouvé sa place. La goutte verte a séché sur sa joue. Le bois de l'étal redevient sec. La poire d'en bas a trouvé sa place, grain de cannelle voyageur.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La poire d'en haut a failli tout cacher. On l'a prise, en bas. Le stand est à nous. Vous avez offert le fruit. La poire d'en bas a trouvé sa place. La goutte verte a séché sur sa joue. Le bois de l'étal redevient sec. La poire d'en bas a trouvé sa place, grain voyageur.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La poire d'en haut a failli tout cacher. On l'a prise, en bas. Le stand est à nous. Vous avez offert le fruit. La poire d'en bas a trouvé sa place. La goutte verte a séché sur sa joue. Le bois de l'étal redevient sec. La poire d'en bas a trouvé sa place, &lt;emphasis level="moderate"&gt;grain de cannelle&lt;/emphasis&gt; voyageur.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La poire d'en haut a failli tout cacher. On l'a prise, en bas. Le stand est à nous. Vous avez offert le fruit. La poire d'en bas a trouvé sa place. La goutte verte a séché sur sa joue. Le bois de l'étal redevient sec. La poire d'en bas a trouvé sa place, grain voyageur.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La poire d'en haut a failli tout cacher. On l'a prise, en bas. Le stand est à nous. Vous avez offert le fruit. La poire d'en bas a trouvé sa place. La goutte verte a séché sur sa joue. Le bois de l'étal redevient sec. La poire d'en bas a trouvé sa place, &lt;emphasis&gt;grain de cannelle&lt;/emphasis&gt; voyageur.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -17337,7 +17342,7 @@
 maman|La poire d'en bas a trouvé sa place.
 narrateur|La goutte verte a séché sur sa joue.
 narrateur|Le bois de l'étal redevient sec.
-narrateur|La poire d'en bas a trouvé sa place, grain voyageur.</t>
+narrateur|La poire d'en bas a trouvé sa place, grain de cannelle voyageur.</t>
         </is>
       </c>
       <c r="AX87" t="inlineStr">
@@ -17363,7 +17368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17434,6 +17439,13 @@
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>